<commit_message>
all updates since last commit
</commit_message>
<xml_diff>
--- a/F0AM-4.3.0.1/Chem/GEOSChem/GC_database_final_UPDATED.xlsx
+++ b/F0AM-4.3.0.1/Chem/GEOSChem/GC_database_final_UPDATED.xlsx
@@ -5,18 +5,19 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\u6044586\AppData\Local\Temp\scp37511\uufs\chpc.utah.edu\common\home\u6044586\python_scripts\species_database\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\u1545774\Documents\GitHub\USOS_shared\F0AM-4.3.0.1\Chem\GEOSChem\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A47ABA2A-C353-4DC7-BACC-E78955CC1F33}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C697B635-6B44-44AE-BD6D-658E78F0B772}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="780" yWindow="780" windowWidth="25755" windowHeight="13680" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-36" yWindow="0" windowWidth="10356" windowHeight="12240" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet2" sheetId="2" r:id="rId1"/>
     <sheet name="Sheet3" sheetId="3" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
+  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -26,6 +27,9 @@
         <xcalcf:feature name="microsoft.com:CNMTM"/>
         <xcalcf:feature name="microsoft.com:LET_WF"/>
       </xcalcf:calcFeatures>
+    </ext>
+    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
+      <xlwcv:version setVersion="1"/>
     </ext>
   </extLst>
 </workbook>
@@ -3681,7 +3685,74 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="9">
+  <dxfs count="18">
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="0" tint="-0.14996795556505021"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF00B050"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF00B050"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="6" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="9" tint="-0.24994659260841701"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="9" tint="-0.24994659260841701"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF0070C0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF0070C0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="4" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FFC00000"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FFC00000"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="5" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <fill>
         <patternFill>
@@ -4048,20 +4119,20 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{51475FDE-34E2-4137-961E-D663FFFF3A49}">
   <dimension ref="A1:T348"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="1" max="1" width="17.5703125" style="12" customWidth="1"/>
-    <col min="2" max="2" width="6.140625" style="12" customWidth="1"/>
-    <col min="3" max="3" width="24.5703125" style="12" customWidth="1"/>
+    <col min="1" max="1" width="17.59765625" style="12" customWidth="1"/>
+    <col min="2" max="2" width="6.1328125" style="12" customWidth="1"/>
+    <col min="3" max="3" width="24.59765625" style="12" customWidth="1"/>
     <col min="4" max="4" width="36" style="17" customWidth="1"/>
-    <col min="5" max="5" width="9.140625" style="12"/>
+    <col min="5" max="5" width="9.1328125" style="12"/>
     <col min="6" max="6" width="50" style="14" customWidth="1"/>
-    <col min="7" max="7" width="11.42578125" style="25" customWidth="1"/>
-    <col min="8" max="8" width="19.5703125" style="21" customWidth="1"/>
-    <col min="12" max="12" width="9.140625" customWidth="1"/>
+    <col min="7" max="7" width="11.3984375" style="25" customWidth="1"/>
+    <col min="8" max="8" width="19.59765625" style="21" customWidth="1"/>
+    <col min="12" max="12" width="9.1328125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:20" s="9" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:20" s="9" customFormat="1" x14ac:dyDescent="0.45">
       <c r="A1" s="11" t="s">
         <v>1105</v>
       </c>
@@ -4087,7 +4158,7 @@
         <v>1126</v>
       </c>
     </row>
-    <row r="2" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A2" s="7" t="s">
         <v>1</v>
       </c>
@@ -4110,7 +4181,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="3" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A3" s="7" t="s">
         <v>6</v>
       </c>
@@ -4130,7 +4201,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="4" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A4" s="7" t="s">
         <v>832</v>
       </c>
@@ -4153,7 +4224,7 @@
         <v>832</v>
       </c>
     </row>
-    <row r="5" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A5" s="7" t="s">
         <v>835</v>
       </c>
@@ -4176,7 +4247,7 @@
       <c r="I5" s="3"/>
       <c r="J5" s="3"/>
     </row>
-    <row r="6" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A6" s="7" t="s">
         <v>838</v>
       </c>
@@ -4196,7 +4267,7 @@
         <v>1112</v>
       </c>
     </row>
-    <row r="7" spans="1:20" s="3" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:20" s="3" customFormat="1" x14ac:dyDescent="0.45">
       <c r="A7" s="7" t="s">
         <v>10</v>
       </c>
@@ -4230,7 +4301,7 @@
       <c r="S7"/>
       <c r="T7"/>
     </row>
-    <row r="8" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A8" s="7" t="s">
         <v>14</v>
       </c>
@@ -4250,7 +4321,7 @@
         <v>1087</v>
       </c>
     </row>
-    <row r="9" spans="1:20" s="3" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:20" s="3" customFormat="1" x14ac:dyDescent="0.45">
       <c r="A9" s="7" t="s">
         <v>18</v>
       </c>
@@ -4284,7 +4355,7 @@
       <c r="S9"/>
       <c r="T9"/>
     </row>
-    <row r="10" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A10" s="7" t="s">
         <v>22</v>
       </c>
@@ -4304,7 +4375,7 @@
         <v>1139</v>
       </c>
     </row>
-    <row r="11" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A11" s="7" t="s">
         <v>842</v>
       </c>
@@ -4321,7 +4392,7 @@
         <v>150.13</v>
       </c>
     </row>
-    <row r="12" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A12" s="7" t="s">
         <v>844</v>
       </c>
@@ -4354,7 +4425,7 @@
       <c r="S12" s="4"/>
       <c r="T12" s="4"/>
     </row>
-    <row r="13" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A13" s="7" t="s">
         <v>846</v>
       </c>
@@ -4374,7 +4445,7 @@
         <v>1130</v>
       </c>
     </row>
-    <row r="14" spans="1:20" s="3" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:20" s="3" customFormat="1" x14ac:dyDescent="0.45">
       <c r="A14" s="7" t="s">
         <v>847</v>
       </c>
@@ -4410,7 +4481,7 @@
       <c r="S14"/>
       <c r="T14"/>
     </row>
-    <row r="15" spans="1:20" s="3" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:20" s="3" customFormat="1" x14ac:dyDescent="0.45">
       <c r="A15" s="1" t="s">
         <v>848</v>
       </c>
@@ -4444,7 +4515,7 @@
       <c r="S15"/>
       <c r="T15"/>
     </row>
-    <row r="16" spans="1:20" s="3" customFormat="1" ht="30" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:20" s="3" customFormat="1" ht="28.5" x14ac:dyDescent="0.45">
       <c r="A16" s="7" t="s">
         <v>24</v>
       </c>
@@ -4474,7 +4545,7 @@
       <c r="S16" s="4"/>
       <c r="T16" s="4"/>
     </row>
-    <row r="17" spans="1:20" s="3" customFormat="1" ht="30" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:20" s="3" customFormat="1" ht="28.5" x14ac:dyDescent="0.45">
       <c r="A17" s="7" t="s">
         <v>851</v>
       </c>
@@ -4500,7 +4571,7 @@
       <c r="I17"/>
       <c r="J17"/>
     </row>
-    <row r="18" spans="1:20" s="3" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:20" s="3" customFormat="1" x14ac:dyDescent="0.45">
       <c r="A18" s="7" t="s">
         <v>853</v>
       </c>
@@ -4532,7 +4603,7 @@
       <c r="S18"/>
       <c r="T18"/>
     </row>
-    <row r="19" spans="1:20" s="4" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:20" s="4" customFormat="1" x14ac:dyDescent="0.45">
       <c r="A19" s="7" t="s">
         <v>855</v>
       </c>
@@ -4564,7 +4635,7 @@
       <c r="S19"/>
       <c r="T19"/>
     </row>
-    <row r="20" spans="1:20" s="4" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:20" s="4" customFormat="1" x14ac:dyDescent="0.45">
       <c r="A20" s="7" t="s">
         <v>857</v>
       </c>
@@ -4596,7 +4667,7 @@
       <c r="S20"/>
       <c r="T20"/>
     </row>
-    <row r="21" spans="1:20" s="4" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:20" s="4" customFormat="1" x14ac:dyDescent="0.45">
       <c r="A21" s="7" t="s">
         <v>860</v>
       </c>
@@ -4630,7 +4701,7 @@
       <c r="S21"/>
       <c r="T21"/>
     </row>
-    <row r="22" spans="1:20" s="4" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:20" s="4" customFormat="1" x14ac:dyDescent="0.45">
       <c r="A22" s="7" t="s">
         <v>863</v>
       </c>
@@ -4662,7 +4733,7 @@
       <c r="S22"/>
       <c r="T22"/>
     </row>
-    <row r="23" spans="1:20" s="3" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:20" s="3" customFormat="1" x14ac:dyDescent="0.45">
       <c r="A23" s="7" t="s">
         <v>27</v>
       </c>
@@ -4698,7 +4769,7 @@
       <c r="S23"/>
       <c r="T23"/>
     </row>
-    <row r="24" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A24" s="7" t="s">
         <v>31</v>
       </c>
@@ -4721,7 +4792,7 @@
         <v>1139</v>
       </c>
     </row>
-    <row r="25" spans="1:20" s="3" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:20" s="3" customFormat="1" x14ac:dyDescent="0.45">
       <c r="A25" s="7" t="s">
         <v>866</v>
       </c>
@@ -4753,7 +4824,7 @@
       <c r="S25"/>
       <c r="T25"/>
     </row>
-    <row r="26" spans="1:20" s="3" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:20" s="3" customFormat="1" x14ac:dyDescent="0.45">
       <c r="A26" s="7" t="s">
         <v>35</v>
       </c>
@@ -4785,7 +4856,7 @@
       <c r="S26"/>
       <c r="T26"/>
     </row>
-    <row r="27" spans="1:20" s="4" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:20" s="4" customFormat="1" x14ac:dyDescent="0.45">
       <c r="A27" s="7" t="s">
         <v>38</v>
       </c>
@@ -4821,7 +4892,7 @@
       <c r="S27"/>
       <c r="T27"/>
     </row>
-    <row r="28" spans="1:20" s="3" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:20" s="3" customFormat="1" x14ac:dyDescent="0.45">
       <c r="A28" s="7" t="s">
         <v>43</v>
       </c>
@@ -4857,7 +4928,7 @@
       <c r="S28"/>
       <c r="T28"/>
     </row>
-    <row r="29" spans="1:20" s="3" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:20" s="3" customFormat="1" x14ac:dyDescent="0.45">
       <c r="A29" s="7" t="s">
         <v>46</v>
       </c>
@@ -4893,7 +4964,7 @@
       <c r="S29"/>
       <c r="T29"/>
     </row>
-    <row r="30" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A30" s="7" t="s">
         <v>50</v>
       </c>
@@ -4913,7 +4984,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="31" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A31" s="7" t="s">
         <v>54</v>
       </c>
@@ -4933,7 +5004,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="32" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A32" s="7" t="s">
         <v>58</v>
       </c>
@@ -4953,7 +5024,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="33" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A33" s="7" t="s">
         <v>62</v>
       </c>
@@ -4976,7 +5047,7 @@
         <v>1139</v>
       </c>
     </row>
-    <row r="34" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A34" s="7" t="s">
         <v>66</v>
       </c>
@@ -4996,7 +5067,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="35" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A35" s="7" t="s">
         <v>871</v>
       </c>
@@ -5013,7 +5084,7 @@
         <v>215.28</v>
       </c>
     </row>
-    <row r="36" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A36" s="7" t="s">
         <v>873</v>
       </c>
@@ -5033,7 +5104,7 @@
       <c r="I36" s="3"/>
       <c r="J36" s="3"/>
     </row>
-    <row r="37" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A37" s="7" t="s">
         <v>876</v>
       </c>
@@ -5051,7 +5122,7 @@
       </c>
       <c r="F37" s="15"/>
     </row>
-    <row r="38" spans="1:20" s="3" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:20" s="3" customFormat="1" x14ac:dyDescent="0.45">
       <c r="A38" s="7" t="s">
         <v>878</v>
       </c>
@@ -5081,7 +5152,7 @@
       <c r="S38"/>
       <c r="T38"/>
     </row>
-    <row r="39" spans="1:20" s="3" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:20" s="3" customFormat="1" x14ac:dyDescent="0.45">
       <c r="A39" s="7" t="s">
         <v>881</v>
       </c>
@@ -5113,7 +5184,7 @@
       <c r="S39"/>
       <c r="T39"/>
     </row>
-    <row r="40" spans="1:20" s="3" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:20" s="3" customFormat="1" x14ac:dyDescent="0.45">
       <c r="A40" s="7" t="s">
         <v>883</v>
       </c>
@@ -5145,7 +5216,7 @@
       <c r="S40"/>
       <c r="T40"/>
     </row>
-    <row r="41" spans="1:20" s="3" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:20" s="3" customFormat="1" x14ac:dyDescent="0.45">
       <c r="A41" s="7" t="s">
         <v>886</v>
       </c>
@@ -5175,7 +5246,7 @@
       <c r="S41"/>
       <c r="T41"/>
     </row>
-    <row r="42" spans="1:20" s="3" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:20" s="3" customFormat="1" x14ac:dyDescent="0.45">
       <c r="A42" s="7" t="s">
         <v>86</v>
       </c>
@@ -5209,7 +5280,7 @@
       <c r="S42" s="5"/>
       <c r="T42" s="5"/>
     </row>
-    <row r="43" spans="1:20" s="3" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:20" s="3" customFormat="1" x14ac:dyDescent="0.45">
       <c r="A43" s="7" t="s">
         <v>89</v>
       </c>
@@ -5233,7 +5304,7 @@
       <c r="I43"/>
       <c r="J43"/>
     </row>
-    <row r="44" spans="1:20" s="3" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:20" s="3" customFormat="1" x14ac:dyDescent="0.45">
       <c r="A44" s="7" t="s">
         <v>92</v>
       </c>
@@ -5257,7 +5328,7 @@
       <c r="I44"/>
       <c r="J44"/>
     </row>
-    <row r="45" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A45" s="7" t="s">
         <v>95</v>
       </c>
@@ -5287,7 +5358,7 @@
       <c r="S45" s="3"/>
       <c r="T45" s="3"/>
     </row>
-    <row r="46" spans="1:20" s="4" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:20" s="4" customFormat="1" x14ac:dyDescent="0.45">
       <c r="A46" s="7" t="s">
         <v>98</v>
       </c>
@@ -5321,7 +5392,7 @@
       <c r="S46" s="6"/>
       <c r="T46" s="6"/>
     </row>
-    <row r="47" spans="1:20" s="3" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:20" s="3" customFormat="1" x14ac:dyDescent="0.45">
       <c r="A47" s="7" t="s">
         <v>101</v>
       </c>
@@ -5355,7 +5426,7 @@
       <c r="S47"/>
       <c r="T47"/>
     </row>
-    <row r="48" spans="1:20" s="3" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:20" s="3" customFormat="1" x14ac:dyDescent="0.45">
       <c r="A48" s="7" t="s">
         <v>70</v>
       </c>
@@ -5389,7 +5460,7 @@
       <c r="S48"/>
       <c r="T48"/>
     </row>
-    <row r="49" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A49" s="7" t="s">
         <v>104</v>
       </c>
@@ -5409,7 +5480,7 @@
         <v>1088</v>
       </c>
     </row>
-    <row r="50" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A50" s="7" t="s">
         <v>106</v>
       </c>
@@ -5429,7 +5500,7 @@
         <v>1088</v>
       </c>
     </row>
-    <row r="51" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A51" s="7" t="s">
         <v>888</v>
       </c>
@@ -5449,7 +5520,7 @@
         <v>1097</v>
       </c>
     </row>
-    <row r="52" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A52" s="7" t="s">
         <v>890</v>
       </c>
@@ -5469,7 +5540,7 @@
       <c r="I52" s="3"/>
       <c r="J52" s="3"/>
     </row>
-    <row r="53" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A53" s="7" t="s">
         <v>893</v>
       </c>
@@ -5492,7 +5563,7 @@
         <v>1136</v>
       </c>
     </row>
-    <row r="54" spans="1:20" ht="30" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A54" s="7" t="s">
         <v>74</v>
       </c>
@@ -5512,7 +5583,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="55" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A55" s="7" t="s">
         <v>78</v>
       </c>
@@ -5535,7 +5606,7 @@
       <c r="I55" s="5"/>
       <c r="J55" s="5"/>
     </row>
-    <row r="56" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A56" s="7" t="s">
         <v>82</v>
       </c>
@@ -5558,7 +5629,7 @@
       <c r="I56" s="3"/>
       <c r="J56" s="3"/>
     </row>
-    <row r="57" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A57" s="7" t="s">
         <v>108</v>
       </c>
@@ -5578,7 +5649,7 @@
         <v>110</v>
       </c>
     </row>
-    <row r="58" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A58" s="7" t="s">
         <v>111</v>
       </c>
@@ -5601,7 +5672,7 @@
       <c r="I58" s="3"/>
       <c r="J58" s="3"/>
     </row>
-    <row r="59" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A59" s="7" t="s">
         <v>114</v>
       </c>
@@ -5624,7 +5695,7 @@
       <c r="I59" s="3"/>
       <c r="J59" s="3"/>
     </row>
-    <row r="60" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A60" s="7" t="s">
         <v>117</v>
       </c>
@@ -5644,7 +5715,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="61" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A61" s="7" t="s">
         <v>895</v>
       </c>
@@ -5667,7 +5738,7 @@
       <c r="I61" s="4"/>
       <c r="J61" s="4"/>
     </row>
-    <row r="62" spans="1:20" ht="30" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:20" ht="28.5" x14ac:dyDescent="0.45">
       <c r="A62" s="7" t="s">
         <v>120</v>
       </c>
@@ -5687,7 +5758,7 @@
         <v>122</v>
       </c>
     </row>
-    <row r="63" spans="1:20" ht="30" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:20" ht="28.5" x14ac:dyDescent="0.45">
       <c r="A63" s="7" t="s">
         <v>123</v>
       </c>
@@ -5717,7 +5788,7 @@
       <c r="S63" s="3"/>
       <c r="T63" s="3"/>
     </row>
-    <row r="64" spans="1:20" s="4" customFormat="1" ht="30" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:20" s="4" customFormat="1" ht="28.5" x14ac:dyDescent="0.45">
       <c r="A64" s="7" t="s">
         <v>898</v>
       </c>
@@ -5751,7 +5822,7 @@
       <c r="S64"/>
       <c r="T64"/>
     </row>
-    <row r="65" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A65" s="7" t="s">
         <v>901</v>
       </c>
@@ -5768,7 +5839,7 @@
         <v>185.27</v>
       </c>
     </row>
-    <row r="66" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A66" s="7" t="s">
         <v>903</v>
       </c>
@@ -5798,7 +5869,7 @@
       <c r="S66" s="3"/>
       <c r="T66" s="3"/>
     </row>
-    <row r="67" spans="1:20" s="3" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:20" s="3" customFormat="1" x14ac:dyDescent="0.45">
       <c r="A67" s="7" t="s">
         <v>125</v>
       </c>
@@ -5822,7 +5893,7 @@
       <c r="I67"/>
       <c r="J67"/>
     </row>
-    <row r="68" spans="1:20" s="3" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:20" s="3" customFormat="1" x14ac:dyDescent="0.45">
       <c r="A68" s="7" t="s">
         <v>128</v>
       </c>
@@ -5844,7 +5915,7 @@
       <c r="G68" s="25"/>
       <c r="H68" s="22"/>
     </row>
-    <row r="69" spans="1:20" s="3" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:20" s="3" customFormat="1" x14ac:dyDescent="0.45">
       <c r="A69" s="7" t="s">
         <v>132</v>
       </c>
@@ -5866,7 +5937,7 @@
       <c r="G69" s="25"/>
       <c r="H69" s="22"/>
     </row>
-    <row r="70" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A70" s="7" t="s">
         <v>136</v>
       </c>
@@ -5886,7 +5957,7 @@
         <v>139</v>
       </c>
     </row>
-    <row r="71" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A71" s="7" t="s">
         <v>140</v>
       </c>
@@ -5906,7 +5977,7 @@
         <v>143</v>
       </c>
     </row>
-    <row r="72" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A72" s="7" t="s">
         <v>144</v>
       </c>
@@ -5926,7 +5997,7 @@
         <v>147</v>
       </c>
     </row>
-    <row r="73" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A73" s="7" t="s">
         <v>148</v>
       </c>
@@ -5946,7 +6017,7 @@
         <v>907</v>
       </c>
     </row>
-    <row r="74" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A74" s="7" t="s">
         <v>150</v>
       </c>
@@ -5966,7 +6037,7 @@
         <v>152</v>
       </c>
     </row>
-    <row r="75" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A75" s="7" t="s">
         <v>153</v>
       </c>
@@ -5986,7 +6057,7 @@
         <v>155</v>
       </c>
     </row>
-    <row r="76" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A76" s="7" t="s">
         <v>156</v>
       </c>
@@ -6006,7 +6077,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="77" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A77" s="7" t="s">
         <v>159</v>
       </c>
@@ -6026,7 +6097,7 @@
         <v>161</v>
       </c>
     </row>
-    <row r="78" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A78" s="7" t="s">
         <v>162</v>
       </c>
@@ -6049,7 +6120,7 @@
       <c r="I78" s="3"/>
       <c r="J78" s="3"/>
     </row>
-    <row r="79" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A79" s="7" t="s">
         <v>165</v>
       </c>
@@ -6079,7 +6150,7 @@
       <c r="S79" s="3"/>
       <c r="T79" s="3"/>
     </row>
-    <row r="80" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A80" s="7" t="s">
         <v>168</v>
       </c>
@@ -6109,7 +6180,7 @@
       <c r="S80" s="3"/>
       <c r="T80" s="3"/>
     </row>
-    <row r="81" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A81" s="7" t="s">
         <v>171</v>
       </c>
@@ -6142,7 +6213,7 @@
       <c r="S81" s="3"/>
       <c r="T81" s="3"/>
     </row>
-    <row r="82" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A82" s="7" t="s">
         <v>174</v>
       </c>
@@ -6172,7 +6243,7 @@
       <c r="S82" s="3"/>
       <c r="T82" s="3"/>
     </row>
-    <row r="83" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A83" s="7" t="s">
         <v>176</v>
       </c>
@@ -6195,7 +6266,7 @@
       <c r="I83" s="3"/>
       <c r="J83" s="3"/>
     </row>
-    <row r="84" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A84" s="7" t="s">
         <v>179</v>
       </c>
@@ -6218,7 +6289,7 @@
       <c r="I84" s="6"/>
       <c r="J84" s="6"/>
     </row>
-    <row r="85" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A85" s="7" t="s">
         <v>182</v>
       </c>
@@ -6238,7 +6309,7 @@
         <v>184</v>
       </c>
     </row>
-    <row r="86" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A86" s="7" t="s">
         <v>185</v>
       </c>
@@ -6261,7 +6332,7 @@
       <c r="I86" s="3"/>
       <c r="J86" s="3"/>
     </row>
-    <row r="87" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A87" s="7" t="s">
         <v>188</v>
       </c>
@@ -6284,7 +6355,7 @@
       <c r="I87" s="3"/>
       <c r="J87" s="3"/>
     </row>
-    <row r="88" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A88" s="7" t="s">
         <v>201</v>
       </c>
@@ -6307,7 +6378,7 @@
       <c r="I88" s="3"/>
       <c r="J88" s="3"/>
     </row>
-    <row r="89" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A89" s="7" t="s">
         <v>204</v>
       </c>
@@ -6327,7 +6398,7 @@
         <v>206</v>
       </c>
     </row>
-    <row r="90" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A90" s="7" t="s">
         <v>207</v>
       </c>
@@ -6350,7 +6421,7 @@
       <c r="I90" s="3"/>
       <c r="J90" s="3"/>
     </row>
-    <row r="91" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A91" s="7" t="s">
         <v>210</v>
       </c>
@@ -6370,7 +6441,7 @@
         <v>212</v>
       </c>
     </row>
-    <row r="92" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A92" s="7" t="s">
         <v>213</v>
       </c>
@@ -6390,7 +6461,7 @@
         <v>215</v>
       </c>
     </row>
-    <row r="93" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A93" s="7" t="s">
         <v>216</v>
       </c>
@@ -6413,7 +6484,7 @@
       <c r="I93" s="3"/>
       <c r="J93" s="3"/>
     </row>
-    <row r="94" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A94" s="7" t="s">
         <v>219</v>
       </c>
@@ -6436,7 +6507,7 @@
       <c r="I94" s="3"/>
       <c r="J94" s="3"/>
     </row>
-    <row r="95" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="95" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A95" s="7" t="s">
         <v>191</v>
       </c>
@@ -6456,7 +6527,7 @@
         <v>193</v>
       </c>
     </row>
-    <row r="96" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="96" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A96" s="7" t="s">
         <v>194</v>
       </c>
@@ -6476,7 +6547,7 @@
         <v>196</v>
       </c>
     </row>
-    <row r="97" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="97" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A97" s="7" t="s">
         <v>197</v>
       </c>
@@ -6496,7 +6567,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="98" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="98" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A98" s="7" t="s">
         <v>222</v>
       </c>
@@ -6519,7 +6590,7 @@
       <c r="I98" s="4"/>
       <c r="J98" s="4"/>
     </row>
-    <row r="99" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="99" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A99" s="7" t="s">
         <v>909</v>
       </c>
@@ -6539,7 +6610,7 @@
         <v>1099</v>
       </c>
     </row>
-    <row r="100" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="100" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A100" s="7" t="s">
         <v>225</v>
       </c>
@@ -6562,7 +6633,7 @@
       <c r="I100" s="3"/>
       <c r="J100" s="3"/>
     </row>
-    <row r="101" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="101" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A101" s="7" t="s">
         <v>229</v>
       </c>
@@ -6582,7 +6653,7 @@
         <v>230</v>
       </c>
     </row>
-    <row r="102" spans="1:20" s="4" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="102" spans="1:20" s="4" customFormat="1" x14ac:dyDescent="0.45">
       <c r="A102" s="7" t="s">
         <v>231</v>
       </c>
@@ -6616,7 +6687,7 @@
       <c r="S102"/>
       <c r="T102"/>
     </row>
-    <row r="103" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="103" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A103" s="7" t="s">
         <v>235</v>
       </c>
@@ -6636,7 +6707,7 @@
         <v>238</v>
       </c>
     </row>
-    <row r="104" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="104" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A104" s="7" t="s">
         <v>239</v>
       </c>
@@ -6659,7 +6730,7 @@
       <c r="I104" s="4"/>
       <c r="J104" s="4"/>
     </row>
-    <row r="105" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="105" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A105" s="7" t="s">
         <v>243</v>
       </c>
@@ -6679,7 +6750,7 @@
         <v>246</v>
       </c>
     </row>
-    <row r="106" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="106" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A106" s="7" t="s">
         <v>247</v>
       </c>
@@ -6699,7 +6770,7 @@
         <v>249</v>
       </c>
     </row>
-    <row r="107" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="107" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A107" s="7" t="s">
         <v>250</v>
       </c>
@@ -6719,7 +6790,7 @@
         <v>253</v>
       </c>
     </row>
-    <row r="108" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="108" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A108" s="7" t="s">
         <v>254</v>
       </c>
@@ -6739,7 +6810,7 @@
         <v>257</v>
       </c>
     </row>
-    <row r="109" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="109" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A109" s="7" t="s">
         <v>913</v>
       </c>
@@ -6759,7 +6830,7 @@
         <v>1139</v>
       </c>
     </row>
-    <row r="110" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="110" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A110" s="7" t="s">
         <v>913</v>
       </c>
@@ -6780,7 +6851,7 @@
       </c>
       <c r="G110" s="32"/>
     </row>
-    <row r="111" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="111" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A111" s="7" t="s">
         <v>915</v>
       </c>
@@ -6803,7 +6874,7 @@
         <v>916</v>
       </c>
     </row>
-    <row r="112" spans="1:20" s="4" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="112" spans="1:20" s="4" customFormat="1" x14ac:dyDescent="0.45">
       <c r="A112" s="7" t="s">
         <v>258</v>
       </c>
@@ -6837,7 +6908,7 @@
       <c r="S112"/>
       <c r="T112"/>
     </row>
-    <row r="113" spans="1:20" s="3" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="113" spans="1:20" s="3" customFormat="1" x14ac:dyDescent="0.45">
       <c r="A113" s="7" t="s">
         <v>261</v>
       </c>
@@ -6869,7 +6940,7 @@
       <c r="S113"/>
       <c r="T113"/>
     </row>
-    <row r="114" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="114" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A114" s="7" t="s">
         <v>264</v>
       </c>
@@ -6889,7 +6960,7 @@
         <v>1092</v>
       </c>
     </row>
-    <row r="115" spans="1:20" s="4" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="115" spans="1:20" s="4" customFormat="1" x14ac:dyDescent="0.45">
       <c r="A115" s="7" t="s">
         <v>266</v>
       </c>
@@ -6923,7 +6994,7 @@
       <c r="S115"/>
       <c r="T115"/>
     </row>
-    <row r="116" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="116" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A116" s="7" t="s">
         <v>270</v>
       </c>
@@ -6953,7 +7024,7 @@
       <c r="S116" s="3"/>
       <c r="T116" s="3"/>
     </row>
-    <row r="117" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="117" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A117" s="7" t="s">
         <v>274</v>
       </c>
@@ -6983,7 +7054,7 @@
       <c r="S117" s="5"/>
       <c r="T117" s="5"/>
     </row>
-    <row r="118" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="118" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A118" s="7" t="s">
         <v>277</v>
       </c>
@@ -7013,7 +7084,7 @@
       <c r="S118" s="5"/>
       <c r="T118" s="5"/>
     </row>
-    <row r="119" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="119" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A119" s="7" t="s">
         <v>281</v>
       </c>
@@ -7043,7 +7114,7 @@
       <c r="S119" s="6"/>
       <c r="T119" s="6"/>
     </row>
-    <row r="120" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="120" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A120" s="7" t="s">
         <v>285</v>
       </c>
@@ -7076,7 +7147,7 @@
       <c r="S120" s="3"/>
       <c r="T120" s="3"/>
     </row>
-    <row r="121" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="121" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A121" s="7" t="s">
         <v>288</v>
       </c>
@@ -7106,7 +7177,7 @@
       <c r="S121" s="3"/>
       <c r="T121" s="3"/>
     </row>
-    <row r="122" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="122" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A122" s="7" t="s">
         <v>921</v>
       </c>
@@ -7136,7 +7207,7 @@
       <c r="S122" s="6"/>
       <c r="T122" s="6"/>
     </row>
-    <row r="123" spans="1:20" s="4" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="123" spans="1:20" s="4" customFormat="1" x14ac:dyDescent="0.45">
       <c r="A123" s="7" t="s">
         <v>291</v>
       </c>
@@ -7170,7 +7241,7 @@
       <c r="S123" s="6"/>
       <c r="T123" s="6"/>
     </row>
-    <row r="124" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="124" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A124" s="7" t="s">
         <v>294</v>
       </c>
@@ -7190,7 +7261,7 @@
         <v>296</v>
       </c>
     </row>
-    <row r="125" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="125" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A125" s="7" t="s">
         <v>297</v>
       </c>
@@ -7210,7 +7281,7 @@
         <v>300</v>
       </c>
     </row>
-    <row r="126" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="126" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A126" s="7" t="s">
         <v>301</v>
       </c>
@@ -7230,7 +7301,7 @@
         <v>304</v>
       </c>
     </row>
-    <row r="127" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="127" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A127" s="7" t="s">
         <v>305</v>
       </c>
@@ -7253,7 +7324,7 @@
       <c r="I127" s="4"/>
       <c r="J127" s="4"/>
     </row>
-    <row r="128" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="128" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A128" s="7" t="s">
         <v>309</v>
       </c>
@@ -7273,7 +7344,7 @@
         <v>312</v>
       </c>
     </row>
-    <row r="129" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="129" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A129" s="7" t="s">
         <v>316</v>
       </c>
@@ -7296,7 +7367,7 @@
       <c r="I129" s="3"/>
       <c r="J129" s="3"/>
     </row>
-    <row r="130" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="130" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A130" s="7" t="s">
         <v>313</v>
       </c>
@@ -7316,7 +7387,7 @@
         <v>315</v>
       </c>
     </row>
-    <row r="131" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="131" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A131" s="7" t="s">
         <v>319</v>
       </c>
@@ -7336,7 +7407,7 @@
         <v>321</v>
       </c>
     </row>
-    <row r="132" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="132" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A132" s="7" t="s">
         <v>322</v>
       </c>
@@ -7359,7 +7430,7 @@
       <c r="I132" s="3"/>
       <c r="J132" s="3"/>
     </row>
-    <row r="133" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="133" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A133" s="7" t="s">
         <v>325</v>
       </c>
@@ -7379,7 +7450,7 @@
         <v>927</v>
       </c>
     </row>
-    <row r="134" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="134" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A134" s="7" t="s">
         <v>327</v>
       </c>
@@ -7399,7 +7470,7 @@
         <v>1143</v>
       </c>
     </row>
-    <row r="135" spans="1:20" s="4" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="135" spans="1:20" s="4" customFormat="1" x14ac:dyDescent="0.45">
       <c r="A135" s="7" t="s">
         <v>329</v>
       </c>
@@ -7433,7 +7504,7 @@
       <c r="S135"/>
       <c r="T135"/>
     </row>
-    <row r="136" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="136" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A136" s="7" t="s">
         <v>332</v>
       </c>
@@ -7463,7 +7534,7 @@
       <c r="S136" s="3"/>
       <c r="T136" s="3"/>
     </row>
-    <row r="137" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="137" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A137" s="7" t="s">
         <v>335</v>
       </c>
@@ -7493,7 +7564,7 @@
       <c r="S137" s="3"/>
       <c r="T137" s="3"/>
     </row>
-    <row r="138" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="138" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A138" s="7" t="s">
         <v>338</v>
       </c>
@@ -7513,7 +7584,7 @@
         <v>340</v>
       </c>
     </row>
-    <row r="139" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="139" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A139" s="7" t="s">
         <v>341</v>
       </c>
@@ -7533,7 +7604,7 @@
         <v>343</v>
       </c>
     </row>
-    <row r="140" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="140" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A140" s="7" t="s">
         <v>344</v>
       </c>
@@ -7553,7 +7624,7 @@
         <v>346</v>
       </c>
     </row>
-    <row r="141" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="141" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A141" s="7" t="s">
         <v>347</v>
       </c>
@@ -7576,7 +7647,7 @@
       <c r="I141" s="6"/>
       <c r="J141" s="6"/>
     </row>
-    <row r="142" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="142" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A142" s="7" t="s">
         <v>350</v>
       </c>
@@ -7590,7 +7661,7 @@
         <v>215</v>
       </c>
     </row>
-    <row r="143" spans="1:20" s="3" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="143" spans="1:20" s="3" customFormat="1" x14ac:dyDescent="0.45">
       <c r="A143" s="7" t="s">
         <v>352</v>
       </c>
@@ -7624,7 +7695,7 @@
       <c r="S143"/>
       <c r="T143"/>
     </row>
-    <row r="144" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="144" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A144" s="7" t="s">
         <v>354</v>
       </c>
@@ -7647,7 +7718,7 @@
       <c r="I144" s="6"/>
       <c r="J144" s="6"/>
     </row>
-    <row r="145" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="145" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A145" s="7" t="s">
         <v>357</v>
       </c>
@@ -7667,7 +7738,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="146" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="146" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A146" s="7" t="s">
         <v>359</v>
       </c>
@@ -7690,7 +7761,7 @@
       <c r="I146" s="6"/>
       <c r="J146" s="6"/>
     </row>
-    <row r="147" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="147" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A147" s="7" t="s">
         <v>361</v>
       </c>
@@ -7710,7 +7781,7 @@
         <v>362</v>
       </c>
     </row>
-    <row r="148" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="148" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A148" s="7" t="s">
         <v>363</v>
       </c>
@@ -7730,7 +7801,7 @@
         <v>364</v>
       </c>
     </row>
-    <row r="149" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="149" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A149" s="7" t="s">
         <v>365</v>
       </c>
@@ -7750,7 +7821,7 @@
         <v>367</v>
       </c>
     </row>
-    <row r="150" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="150" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A150" s="7" t="s">
         <v>16</v>
       </c>
@@ -7770,7 +7841,7 @@
         <v>369</v>
       </c>
     </row>
-    <row r="151" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="151" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A151" s="7" t="s">
         <v>370</v>
       </c>
@@ -7793,7 +7864,7 @@
       <c r="I151" s="3"/>
       <c r="J151" s="3"/>
     </row>
-    <row r="152" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="152" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A152" s="7" t="s">
         <v>373</v>
       </c>
@@ -7816,7 +7887,7 @@
       <c r="I152" s="3"/>
       <c r="J152" s="3"/>
     </row>
-    <row r="153" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="153" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A153" s="7" t="s">
         <v>376</v>
       </c>
@@ -7846,7 +7917,7 @@
       <c r="S153" s="3"/>
       <c r="T153" s="3"/>
     </row>
-    <row r="154" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="154" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A154" s="7" t="s">
         <v>379</v>
       </c>
@@ -7879,7 +7950,7 @@
       <c r="S154" s="5"/>
       <c r="T154" s="5"/>
     </row>
-    <row r="155" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="155" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A155" s="7" t="s">
         <v>382</v>
       </c>
@@ -7909,7 +7980,7 @@
       <c r="S155" s="3"/>
       <c r="T155" s="3"/>
     </row>
-    <row r="156" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="156" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A156" s="7" t="s">
         <v>385</v>
       </c>
@@ -7939,7 +8010,7 @@
       <c r="S156" s="5"/>
       <c r="T156" s="5"/>
     </row>
-    <row r="157" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="157" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A157" s="7" t="s">
         <v>388</v>
       </c>
@@ -7969,7 +8040,7 @@
       <c r="S157" s="5"/>
       <c r="T157" s="5"/>
     </row>
-    <row r="158" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="158" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A158" s="7" t="s">
         <v>398</v>
       </c>
@@ -7999,7 +8070,7 @@
       <c r="S158" s="3"/>
       <c r="T158" s="3"/>
     </row>
-    <row r="159" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="159" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A159" s="7" t="s">
         <v>391</v>
       </c>
@@ -8022,7 +8093,7 @@
       <c r="I159" s="6"/>
       <c r="J159" s="6"/>
     </row>
-    <row r="160" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="160" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A160" s="7" t="s">
         <v>394</v>
       </c>
@@ -8045,7 +8116,7 @@
       <c r="I160" s="3"/>
       <c r="J160" s="3"/>
     </row>
-    <row r="161" spans="1:20" ht="30" x14ac:dyDescent="0.25">
+    <row r="161" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A161" s="7" t="s">
         <v>396</v>
       </c>
@@ -8068,7 +8139,7 @@
       <c r="I161" s="3"/>
       <c r="J161" s="3"/>
     </row>
-    <row r="162" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="162" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A162" s="7" t="s">
         <v>401</v>
       </c>
@@ -8088,7 +8159,7 @@
         <v>402</v>
       </c>
     </row>
-    <row r="163" spans="1:20" ht="30" x14ac:dyDescent="0.25">
+    <row r="163" spans="1:20" ht="28.5" x14ac:dyDescent="0.45">
       <c r="A163" s="7" t="s">
         <v>403</v>
       </c>
@@ -8108,7 +8179,7 @@
         <v>405</v>
       </c>
     </row>
-    <row r="164" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="164" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A164" s="7" t="s">
         <v>406</v>
       </c>
@@ -8138,7 +8209,7 @@
       <c r="S164" s="3"/>
       <c r="T164" s="3"/>
     </row>
-    <row r="165" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="165" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A165" s="7" t="s">
         <v>409</v>
       </c>
@@ -8161,7 +8232,7 @@
       <c r="I165" s="3"/>
       <c r="J165" s="3"/>
     </row>
-    <row r="166" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="166" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A166" s="7" t="s">
         <v>411</v>
       </c>
@@ -8194,7 +8265,7 @@
       <c r="S166" s="3"/>
       <c r="T166" s="3"/>
     </row>
-    <row r="167" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="167" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A167" s="7" t="s">
         <v>414</v>
       </c>
@@ -8227,7 +8298,7 @@
       <c r="S167" s="3"/>
       <c r="T167" s="3"/>
     </row>
-    <row r="168" spans="1:20" ht="30" x14ac:dyDescent="0.25">
+    <row r="168" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A168" s="7" t="s">
         <v>416</v>
       </c>
@@ -8260,7 +8331,7 @@
       <c r="S168" s="4"/>
       <c r="T168" s="4"/>
     </row>
-    <row r="169" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="169" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A169" s="7" t="s">
         <v>417</v>
       </c>
@@ -8290,7 +8361,7 @@
       <c r="S169" s="4"/>
       <c r="T169" s="4"/>
     </row>
-    <row r="170" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="170" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A170" s="7" t="s">
         <v>419</v>
       </c>
@@ -8313,7 +8384,7 @@
       <c r="I170" s="3"/>
       <c r="J170" s="3"/>
     </row>
-    <row r="171" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="171" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A171" s="7" t="s">
         <v>423</v>
       </c>
@@ -8333,7 +8404,7 @@
         <v>422</v>
       </c>
     </row>
-    <row r="172" spans="1:20" ht="30" x14ac:dyDescent="0.25">
+    <row r="172" spans="1:20" ht="28.5" x14ac:dyDescent="0.45">
       <c r="A172" s="7" t="s">
         <v>424</v>
       </c>
@@ -8353,7 +8424,7 @@
         <v>425</v>
       </c>
     </row>
-    <row r="173" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="173" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A173" s="7" t="s">
         <v>426</v>
       </c>
@@ -8373,7 +8444,7 @@
         <v>427</v>
       </c>
     </row>
-    <row r="174" spans="1:20" ht="30" x14ac:dyDescent="0.25">
+    <row r="174" spans="1:20" ht="28.5" x14ac:dyDescent="0.45">
       <c r="A174" s="7" t="s">
         <v>428</v>
       </c>
@@ -8393,7 +8464,7 @@
         <v>429</v>
       </c>
     </row>
-    <row r="175" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="175" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A175" s="7" t="s">
         <v>430</v>
       </c>
@@ -8413,7 +8484,7 @@
         <v>431</v>
       </c>
     </row>
-    <row r="176" spans="1:20" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="176" spans="1:20" ht="16.5" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A176" s="7" t="s">
         <v>432</v>
       </c>
@@ -8433,7 +8504,7 @@
         <v>434</v>
       </c>
     </row>
-    <row r="177" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="177" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A177" s="7" t="s">
         <v>435</v>
       </c>
@@ -8453,7 +8524,7 @@
         <v>436</v>
       </c>
     </row>
-    <row r="178" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="178" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A178" s="7" t="s">
         <v>437</v>
       </c>
@@ -8473,7 +8544,7 @@
         <v>438</v>
       </c>
     </row>
-    <row r="179" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="179" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A179" s="7" t="s">
         <v>439</v>
       </c>
@@ -8493,7 +8564,7 @@
         <v>440</v>
       </c>
     </row>
-    <row r="180" spans="1:20" ht="30" x14ac:dyDescent="0.25">
+    <row r="180" spans="1:20" ht="28.5" x14ac:dyDescent="0.45">
       <c r="A180" s="7" t="s">
         <v>441</v>
       </c>
@@ -8513,7 +8584,7 @@
         <v>443</v>
       </c>
     </row>
-    <row r="181" spans="1:20" ht="30" x14ac:dyDescent="0.25">
+    <row r="181" spans="1:20" ht="28.5" x14ac:dyDescent="0.45">
       <c r="A181" s="7" t="s">
         <v>444</v>
       </c>
@@ -8533,7 +8604,7 @@
         <v>445</v>
       </c>
     </row>
-    <row r="182" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="182" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A182" s="7" t="s">
         <v>446</v>
       </c>
@@ -8563,7 +8634,7 @@
       <c r="S182" s="3"/>
       <c r="T182" s="3"/>
     </row>
-    <row r="183" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="183" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A183" s="7" t="s">
         <v>449</v>
       </c>
@@ -8583,7 +8654,7 @@
         <v>450</v>
       </c>
     </row>
-    <row r="184" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="184" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A184" s="7" t="s">
         <v>451</v>
       </c>
@@ -8613,7 +8684,7 @@
       <c r="S184" s="3"/>
       <c r="T184" s="3"/>
     </row>
-    <row r="185" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="185" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A185" s="7" t="s">
         <v>454</v>
       </c>
@@ -8633,7 +8704,7 @@
         <v>455</v>
       </c>
     </row>
-    <row r="186" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="186" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A186" s="7" t="s">
         <v>456</v>
       </c>
@@ -8653,7 +8724,7 @@
         <v>457</v>
       </c>
     </row>
-    <row r="187" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="187" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A187" s="7" t="s">
         <v>458</v>
       </c>
@@ -8676,7 +8747,7 @@
       <c r="I187" s="6"/>
       <c r="J187" s="6"/>
     </row>
-    <row r="188" spans="1:20" ht="30" x14ac:dyDescent="0.25">
+    <row r="188" spans="1:20" ht="28.5" x14ac:dyDescent="0.45">
       <c r="A188" s="7" t="s">
         <v>462</v>
       </c>
@@ -8690,7 +8761,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="189" spans="1:20" s="3" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="189" spans="1:20" s="3" customFormat="1" x14ac:dyDescent="0.45">
       <c r="A189" s="7" t="s">
         <v>461</v>
       </c>
@@ -8714,7 +8785,7 @@
       <c r="I189"/>
       <c r="J189"/>
     </row>
-    <row r="190" spans="1:20" ht="30" x14ac:dyDescent="0.25">
+    <row r="190" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A190" s="7" t="s">
         <v>464</v>
       </c>
@@ -8744,7 +8815,7 @@
       <c r="S190" s="3"/>
       <c r="T190" s="3"/>
     </row>
-    <row r="191" spans="1:20" ht="30" x14ac:dyDescent="0.25">
+    <row r="191" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A191" s="7" t="s">
         <v>467</v>
       </c>
@@ -8774,7 +8845,7 @@
       <c r="S191" s="3"/>
       <c r="T191" s="3"/>
     </row>
-    <row r="192" spans="1:20" ht="30" x14ac:dyDescent="0.25">
+    <row r="192" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A192" s="7" t="s">
         <v>469</v>
       </c>
@@ -8804,7 +8875,7 @@
       <c r="S192" s="3"/>
       <c r="T192" s="3"/>
     </row>
-    <row r="193" spans="1:20" ht="30" x14ac:dyDescent="0.25">
+    <row r="193" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A193" s="7" t="s">
         <v>471</v>
       </c>
@@ -8834,7 +8905,7 @@
       <c r="S193" s="3"/>
       <c r="T193" s="3"/>
     </row>
-    <row r="194" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="194" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A194" s="7" t="s">
         <v>474</v>
       </c>
@@ -8867,7 +8938,7 @@
       <c r="S194" s="4"/>
       <c r="T194" s="4"/>
     </row>
-    <row r="195" spans="1:20" ht="30" x14ac:dyDescent="0.25">
+    <row r="195" spans="1:20" ht="28.5" x14ac:dyDescent="0.45">
       <c r="A195" s="7" t="s">
         <v>477</v>
       </c>
@@ -8894,7 +8965,7 @@
       <c r="S195" s="4"/>
       <c r="T195" s="4"/>
     </row>
-    <row r="196" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="196" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A196" s="7" t="s">
         <v>480</v>
       </c>
@@ -8924,7 +8995,7 @@
       <c r="S196" s="3"/>
       <c r="T196" s="3"/>
     </row>
-    <row r="197" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="197" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A197" s="7" t="s">
         <v>483</v>
       </c>
@@ -8944,7 +9015,7 @@
         <v>485</v>
       </c>
     </row>
-    <row r="198" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="198" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A198" s="7" t="s">
         <v>487</v>
       </c>
@@ -8974,7 +9045,7 @@
       <c r="S198" s="3"/>
       <c r="T198" s="3"/>
     </row>
-    <row r="199" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="199" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A199" s="7" t="s">
         <v>491</v>
       </c>
@@ -9004,7 +9075,7 @@
       <c r="S199" s="3"/>
       <c r="T199" s="3"/>
     </row>
-    <row r="200" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="200" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A200" s="7" t="s">
         <v>493</v>
       </c>
@@ -9034,7 +9105,7 @@
       <c r="S200" s="4"/>
       <c r="T200" s="4"/>
     </row>
-    <row r="201" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="201" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A201" s="7" t="s">
         <v>495</v>
       </c>
@@ -9064,7 +9135,7 @@
       <c r="S201" s="3"/>
       <c r="T201" s="3"/>
     </row>
-    <row r="202" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="202" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A202" s="7" t="s">
         <v>498</v>
       </c>
@@ -9097,7 +9168,7 @@
       <c r="S202" s="3"/>
       <c r="T202" s="3"/>
     </row>
-    <row r="203" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="203" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A203" s="7" t="s">
         <v>500</v>
       </c>
@@ -9117,7 +9188,7 @@
         <v>501</v>
       </c>
     </row>
-    <row r="204" spans="1:20" ht="30" x14ac:dyDescent="0.25">
+    <row r="204" spans="1:20" ht="28.5" x14ac:dyDescent="0.45">
       <c r="A204" s="7" t="s">
         <v>502</v>
       </c>
@@ -9137,7 +9208,7 @@
         <v>503</v>
       </c>
     </row>
-    <row r="205" spans="1:20" ht="30" x14ac:dyDescent="0.25">
+    <row r="205" spans="1:20" ht="28.5" x14ac:dyDescent="0.45">
       <c r="A205" s="7" t="s">
         <v>504</v>
       </c>
@@ -9157,7 +9228,7 @@
         <v>505</v>
       </c>
     </row>
-    <row r="206" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="206" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A206" s="7" t="s">
         <v>506</v>
       </c>
@@ -9174,7 +9245,7 @@
         <v>101.09</v>
       </c>
     </row>
-    <row r="207" spans="1:20" s="3" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="207" spans="1:20" s="3" customFormat="1" x14ac:dyDescent="0.45">
       <c r="A207" s="7" t="s">
         <v>975</v>
       </c>
@@ -9208,7 +9279,7 @@
       <c r="S207"/>
       <c r="T207"/>
     </row>
-    <row r="208" spans="1:20" s="5" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="208" spans="1:20" s="5" customFormat="1" x14ac:dyDescent="0.45">
       <c r="A208" s="7" t="s">
         <v>979</v>
       </c>
@@ -9240,7 +9311,7 @@
       <c r="S208"/>
       <c r="T208"/>
     </row>
-    <row r="209" spans="1:20" s="5" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="209" spans="1:20" s="5" customFormat="1" x14ac:dyDescent="0.45">
       <c r="A209" s="7" t="s">
         <v>983</v>
       </c>
@@ -9274,7 +9345,7 @@
       <c r="S209" s="3"/>
       <c r="T209" s="3"/>
     </row>
-    <row r="210" spans="1:20" s="5" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="210" spans="1:20" s="5" customFormat="1" x14ac:dyDescent="0.45">
       <c r="A210" s="7" t="s">
         <v>985</v>
       </c>
@@ -9306,7 +9377,7 @@
       <c r="S210" s="3"/>
       <c r="T210" s="3"/>
     </row>
-    <row r="211" spans="1:20" s="3" customFormat="1" ht="30" x14ac:dyDescent="0.25">
+    <row r="211" spans="1:20" s="3" customFormat="1" x14ac:dyDescent="0.45">
       <c r="A211" s="7" t="s">
         <v>987</v>
       </c>
@@ -9326,7 +9397,7 @@
       <c r="G211" s="25"/>
       <c r="H211" s="22"/>
     </row>
-    <row r="212" spans="1:20" s="3" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="212" spans="1:20" s="3" customFormat="1" x14ac:dyDescent="0.45">
       <c r="A212" s="7" t="s">
         <v>989</v>
       </c>
@@ -9346,7 +9417,7 @@
       <c r="G212" s="25"/>
       <c r="H212" s="22"/>
     </row>
-    <row r="213" spans="1:20" s="3" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="213" spans="1:20" s="3" customFormat="1" x14ac:dyDescent="0.45">
       <c r="A213" s="7" t="s">
         <v>509</v>
       </c>
@@ -9368,7 +9439,7 @@
       <c r="G213" s="25"/>
       <c r="H213" s="22"/>
     </row>
-    <row r="214" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="214" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A214" s="7" t="s">
         <v>513</v>
       </c>
@@ -9398,7 +9469,7 @@
       <c r="S214" s="3"/>
       <c r="T214" s="3"/>
     </row>
-    <row r="215" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="215" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A215" s="7" t="s">
         <v>992</v>
       </c>
@@ -9428,7 +9499,7 @@
       <c r="S215" s="3"/>
       <c r="T215" s="3"/>
     </row>
-    <row r="216" spans="1:20" s="5" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="216" spans="1:20" s="5" customFormat="1" x14ac:dyDescent="0.45">
       <c r="A216" s="7" t="s">
         <v>994</v>
       </c>
@@ -9460,7 +9531,7 @@
       <c r="S216"/>
       <c r="T216"/>
     </row>
-    <row r="217" spans="1:20" s="3" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="217" spans="1:20" s="3" customFormat="1" x14ac:dyDescent="0.45">
       <c r="A217" s="7" t="s">
         <v>996</v>
       </c>
@@ -9494,7 +9565,7 @@
       <c r="S217" s="4"/>
       <c r="T217" s="4"/>
     </row>
-    <row r="218" spans="1:20" s="5" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="218" spans="1:20" s="5" customFormat="1" x14ac:dyDescent="0.45">
       <c r="A218" s="7" t="s">
         <v>1000</v>
       </c>
@@ -9526,7 +9597,7 @@
       <c r="S218" s="3"/>
       <c r="T218" s="3"/>
     </row>
-    <row r="219" spans="1:20" s="3" customFormat="1" ht="30" x14ac:dyDescent="0.25">
+    <row r="219" spans="1:20" s="3" customFormat="1" ht="28.5" x14ac:dyDescent="0.45">
       <c r="A219" s="7" t="s">
         <v>516</v>
       </c>
@@ -9548,7 +9619,7 @@
       <c r="I219"/>
       <c r="J219"/>
     </row>
-    <row r="220" spans="1:20" s="6" customFormat="1" ht="30" x14ac:dyDescent="0.25">
+    <row r="220" spans="1:20" s="6" customFormat="1" ht="28.5" x14ac:dyDescent="0.45">
       <c r="A220" s="7" t="s">
         <v>518</v>
       </c>
@@ -9580,7 +9651,7 @@
       <c r="S220"/>
       <c r="T220"/>
     </row>
-    <row r="221" spans="1:20" s="6" customFormat="1" ht="30" x14ac:dyDescent="0.25">
+    <row r="221" spans="1:20" s="6" customFormat="1" ht="28.5" x14ac:dyDescent="0.45">
       <c r="A221" s="7" t="s">
         <v>520</v>
       </c>
@@ -9612,7 +9683,7 @@
       <c r="S221"/>
       <c r="T221"/>
     </row>
-    <row r="222" spans="1:20" s="6" customFormat="1" ht="30" x14ac:dyDescent="0.25">
+    <row r="222" spans="1:20" s="6" customFormat="1" ht="28.5" x14ac:dyDescent="0.45">
       <c r="A222" s="7" t="s">
         <v>522</v>
       </c>
@@ -9644,7 +9715,7 @@
       <c r="S222"/>
       <c r="T222"/>
     </row>
-    <row r="223" spans="1:20" s="6" customFormat="1" ht="30" x14ac:dyDescent="0.25">
+    <row r="223" spans="1:20" s="6" customFormat="1" ht="28.5" x14ac:dyDescent="0.45">
       <c r="A223" s="7" t="s">
         <v>524</v>
       </c>
@@ -9676,7 +9747,7 @@
       <c r="S223"/>
       <c r="T223"/>
     </row>
-    <row r="224" spans="1:20" s="6" customFormat="1" ht="30" x14ac:dyDescent="0.25">
+    <row r="224" spans="1:20" s="6" customFormat="1" ht="28.5" x14ac:dyDescent="0.45">
       <c r="A224" s="7" t="s">
         <v>526</v>
       </c>
@@ -9708,7 +9779,7 @@
       <c r="S224"/>
       <c r="T224"/>
     </row>
-    <row r="225" spans="1:20" s="6" customFormat="1" ht="30" x14ac:dyDescent="0.25">
+    <row r="225" spans="1:20" s="6" customFormat="1" ht="28.5" x14ac:dyDescent="0.45">
       <c r="A225" s="7" t="s">
         <v>528</v>
       </c>
@@ -9740,7 +9811,7 @@
       <c r="S225"/>
       <c r="T225"/>
     </row>
-    <row r="226" spans="1:20" s="3" customFormat="1" ht="30" x14ac:dyDescent="0.25">
+    <row r="226" spans="1:20" s="3" customFormat="1" ht="28.5" x14ac:dyDescent="0.45">
       <c r="A226" s="7" t="s">
         <v>531</v>
       </c>
@@ -9772,7 +9843,7 @@
       <c r="S226"/>
       <c r="T226"/>
     </row>
-    <row r="227" spans="1:20" s="3" customFormat="1" ht="30" x14ac:dyDescent="0.25">
+    <row r="227" spans="1:20" s="3" customFormat="1" ht="28.5" x14ac:dyDescent="0.45">
       <c r="A227" s="7" t="s">
         <v>533</v>
       </c>
@@ -9804,7 +9875,7 @@
       <c r="S227" s="4"/>
       <c r="T227" s="4"/>
     </row>
-    <row r="228" spans="1:20" s="6" customFormat="1" ht="30" x14ac:dyDescent="0.25">
+    <row r="228" spans="1:20" s="6" customFormat="1" ht="28.5" x14ac:dyDescent="0.45">
       <c r="A228" s="7" t="s">
         <v>535</v>
       </c>
@@ -9836,7 +9907,7 @@
       <c r="S228"/>
       <c r="T228"/>
     </row>
-    <row r="229" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="229" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.45">
       <c r="A229" s="7" t="s">
         <v>537</v>
       </c>
@@ -9870,7 +9941,7 @@
       <c r="S229"/>
       <c r="T229"/>
     </row>
-    <row r="230" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="230" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A230" s="7" t="s">
         <v>540</v>
       </c>
@@ -9900,7 +9971,7 @@
       <c r="S230" s="3"/>
       <c r="T230" s="3"/>
     </row>
-    <row r="231" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="231" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A231" s="7" t="s">
         <v>542</v>
       </c>
@@ -9936,7 +10007,7 @@
       <c r="S231" s="3"/>
       <c r="T231" s="3"/>
     </row>
-    <row r="232" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="232" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A232" s="7" t="s">
         <v>546</v>
       </c>
@@ -9966,7 +10037,7 @@
       <c r="S232" s="3"/>
       <c r="T232" s="3"/>
     </row>
-    <row r="233" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="233" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A233" s="7" t="s">
         <v>552</v>
       </c>
@@ -9986,7 +10057,7 @@
         <v>555</v>
       </c>
     </row>
-    <row r="234" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="234" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A234" s="7" t="s">
         <v>557</v>
       </c>
@@ -10006,7 +10077,7 @@
         <v>1008</v>
       </c>
     </row>
-    <row r="235" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="235" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A235" s="7" t="s">
         <v>558</v>
       </c>
@@ -10026,7 +10097,7 @@
         <v>559</v>
       </c>
     </row>
-    <row r="236" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="236" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A236" s="7" t="s">
         <v>560</v>
       </c>
@@ -10049,7 +10120,7 @@
       <c r="I236" s="4"/>
       <c r="J236" s="4"/>
     </row>
-    <row r="237" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="237" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A237" s="7" t="s">
         <v>562</v>
       </c>
@@ -10069,7 +10140,7 @@
         <v>563</v>
       </c>
     </row>
-    <row r="238" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="238" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A238" s="7" t="s">
         <v>564</v>
       </c>
@@ -10089,7 +10160,7 @@
         <v>565</v>
       </c>
     </row>
-    <row r="239" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="239" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A239" s="7" t="s">
         <v>566</v>
       </c>
@@ -10109,7 +10180,7 @@
         <v>567</v>
       </c>
     </row>
-    <row r="240" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="240" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A240" s="7" t="s">
         <v>568</v>
       </c>
@@ -10129,7 +10200,7 @@
         <v>570</v>
       </c>
     </row>
-    <row r="241" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="241" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A241" s="7" t="s">
         <v>571</v>
       </c>
@@ -10152,7 +10223,7 @@
         <v>1139</v>
       </c>
     </row>
-    <row r="242" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="242" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A242" s="7" t="s">
         <v>575</v>
       </c>
@@ -10172,7 +10243,7 @@
         <v>577</v>
       </c>
     </row>
-    <row r="243" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="243" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A243" s="7" t="s">
         <v>1015</v>
       </c>
@@ -10186,7 +10257,7 @@
         <v>105.07</v>
       </c>
     </row>
-    <row r="244" spans="1:20" s="3" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="244" spans="1:20" s="3" customFormat="1" x14ac:dyDescent="0.45">
       <c r="A244" s="7" t="s">
         <v>1016</v>
       </c>
@@ -10218,7 +10289,7 @@
       <c r="S244"/>
       <c r="T244"/>
     </row>
-    <row r="245" spans="1:20" s="3" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="245" spans="1:20" s="3" customFormat="1" x14ac:dyDescent="0.45">
       <c r="A245" s="7" t="s">
         <v>578</v>
       </c>
@@ -10252,7 +10323,7 @@
       <c r="S245"/>
       <c r="T245"/>
     </row>
-    <row r="246" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="246" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A246" s="7" t="s">
         <v>583</v>
       </c>
@@ -10272,7 +10343,7 @@
         <v>584</v>
       </c>
     </row>
-    <row r="247" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="247" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A247" s="7" t="s">
         <v>585</v>
       </c>
@@ -10295,7 +10366,7 @@
       <c r="I247" s="3"/>
       <c r="J247" s="3"/>
     </row>
-    <row r="248" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="248" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A248" s="7" t="s">
         <v>589</v>
       </c>
@@ -10318,7 +10389,7 @@
       <c r="I248" s="3"/>
       <c r="J248" s="3"/>
     </row>
-    <row r="249" spans="1:20" ht="30" x14ac:dyDescent="0.25">
+    <row r="249" spans="1:20" ht="28.5" x14ac:dyDescent="0.45">
       <c r="A249" s="7" t="s">
         <v>593</v>
       </c>
@@ -10335,7 +10406,7 @@
         <v>595</v>
       </c>
     </row>
-    <row r="250" spans="1:20" ht="30" x14ac:dyDescent="0.25">
+    <row r="250" spans="1:20" ht="28.5" x14ac:dyDescent="0.45">
       <c r="A250" s="7" t="s">
         <v>596</v>
       </c>
@@ -10355,7 +10426,7 @@
         <v>598</v>
       </c>
     </row>
-    <row r="251" spans="1:20" ht="30" x14ac:dyDescent="0.25">
+    <row r="251" spans="1:20" ht="28.5" x14ac:dyDescent="0.45">
       <c r="A251" s="7" t="s">
         <v>599</v>
       </c>
@@ -10375,7 +10446,7 @@
         <v>600</v>
       </c>
     </row>
-    <row r="252" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="252" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A252" s="7" t="s">
         <v>601</v>
       </c>
@@ -10398,7 +10469,7 @@
       <c r="I252" s="3"/>
       <c r="J252" s="3"/>
     </row>
-    <row r="253" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="253" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A253" s="7" t="s">
         <v>605</v>
       </c>
@@ -10421,7 +10492,7 @@
       <c r="I253" s="3"/>
       <c r="J253" s="3"/>
     </row>
-    <row r="254" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="254" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A254" s="7" t="s">
         <v>607</v>
       </c>
@@ -10441,7 +10512,7 @@
         <v>609</v>
       </c>
     </row>
-    <row r="255" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="255" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A255" s="7" t="s">
         <v>612</v>
       </c>
@@ -10461,7 +10532,7 @@
         <v>614</v>
       </c>
     </row>
-    <row r="256" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="256" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A256" s="7" t="s">
         <v>615</v>
       </c>
@@ -10483,7 +10554,7 @@
       </c>
       <c r="J256" s="3"/>
     </row>
-    <row r="257" spans="1:20" ht="30" x14ac:dyDescent="0.25">
+    <row r="257" spans="1:20" ht="28.5" x14ac:dyDescent="0.45">
       <c r="A257" s="7" t="s">
         <v>617</v>
       </c>
@@ -10505,7 +10576,7 @@
       </c>
       <c r="J257" s="3"/>
     </row>
-    <row r="258" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="258" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A258" s="7" t="s">
         <v>619</v>
       </c>
@@ -10525,7 +10596,7 @@
         <v>621</v>
       </c>
     </row>
-    <row r="259" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="259" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A259" s="7" t="s">
         <v>622</v>
       </c>
@@ -10545,7 +10616,7 @@
         <v>624</v>
       </c>
     </row>
-    <row r="260" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="260" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A260" s="7" t="s">
         <v>625</v>
       </c>
@@ -10565,7 +10636,7 @@
         <v>927</v>
       </c>
     </row>
-    <row r="261" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="261" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A261" s="7" t="s">
         <v>626</v>
       </c>
@@ -10585,7 +10656,7 @@
         <v>927</v>
       </c>
     </row>
-    <row r="262" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="262" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A262" s="7" t="s">
         <v>627</v>
       </c>
@@ -10605,7 +10676,7 @@
         <v>629</v>
       </c>
     </row>
-    <row r="263" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="263" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A263" s="7" t="s">
         <v>630</v>
       </c>
@@ -10625,7 +10696,7 @@
         <v>631</v>
       </c>
     </row>
-    <row r="264" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="264" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A264" s="7" t="s">
         <v>632</v>
       </c>
@@ -10645,7 +10716,7 @@
         <v>633</v>
       </c>
     </row>
-    <row r="265" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="265" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A265" s="7" t="s">
         <v>634</v>
       </c>
@@ -10675,7 +10746,7 @@
       <c r="S265" s="4"/>
       <c r="T265" s="4"/>
     </row>
-    <row r="266" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="266" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A266" s="7" t="s">
         <v>1032</v>
       </c>
@@ -10692,7 +10763,7 @@
         <v>186.28</v>
       </c>
     </row>
-    <row r="267" spans="1:20" s="3" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="267" spans="1:20" s="3" customFormat="1" x14ac:dyDescent="0.45">
       <c r="A267" s="7" t="s">
         <v>638</v>
       </c>
@@ -10726,7 +10797,7 @@
       <c r="S267"/>
       <c r="T267"/>
     </row>
-    <row r="268" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="268" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A268" s="7" t="s">
         <v>641</v>
       </c>
@@ -10746,7 +10817,7 @@
         <v>643</v>
       </c>
     </row>
-    <row r="269" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="269" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A269" s="7" t="s">
         <v>644</v>
       </c>
@@ -10766,7 +10837,7 @@
         <v>646</v>
       </c>
     </row>
-    <row r="270" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="270" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A270" s="7" t="s">
         <v>647</v>
       </c>
@@ -10796,7 +10867,7 @@
       <c r="S270" s="4"/>
       <c r="T270" s="4"/>
     </row>
-    <row r="271" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="271" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A271" s="7" t="s">
         <v>650</v>
       </c>
@@ -10816,7 +10887,7 @@
         <v>653</v>
       </c>
     </row>
-    <row r="272" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="272" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A272" s="7" t="s">
         <v>654</v>
       </c>
@@ -10836,7 +10907,7 @@
         <v>657</v>
       </c>
     </row>
-    <row r="273" spans="1:20" ht="30" x14ac:dyDescent="0.25">
+    <row r="273" spans="1:20" ht="28.5" x14ac:dyDescent="0.45">
       <c r="A273" s="7" t="s">
         <v>658</v>
       </c>
@@ -10859,7 +10930,7 @@
       <c r="I273" s="3"/>
       <c r="J273" s="3"/>
     </row>
-    <row r="274" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="274" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A274" s="7" t="s">
         <v>660</v>
       </c>
@@ -10882,7 +10953,7 @@
       <c r="I274" s="3"/>
       <c r="J274" s="3"/>
     </row>
-    <row r="275" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="275" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A275" s="7" t="s">
         <v>663</v>
       </c>
@@ -10902,7 +10973,7 @@
         <v>665</v>
       </c>
     </row>
-    <row r="276" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="276" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A276" s="7" t="s">
         <v>656</v>
       </c>
@@ -10922,7 +10993,7 @@
         <v>667</v>
       </c>
     </row>
-    <row r="277" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="277" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A277" s="7" t="s">
         <v>668</v>
       </c>
@@ -10957,7 +11028,7 @@
       <c r="S277" s="4"/>
       <c r="T277" s="4"/>
     </row>
-    <row r="278" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="278" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A278" s="7" t="s">
         <v>672</v>
       </c>
@@ -10977,7 +11048,7 @@
         <v>674</v>
       </c>
     </row>
-    <row r="279" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="279" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A279" s="7" t="s">
         <v>675</v>
       </c>
@@ -10997,7 +11068,7 @@
         <v>678</v>
       </c>
     </row>
-    <row r="280" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="280" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A280" s="7" t="s">
         <v>283</v>
       </c>
@@ -11027,7 +11098,7 @@
       <c r="S280" s="3"/>
       <c r="T280" s="3"/>
     </row>
-    <row r="281" spans="1:20" s="3" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="281" spans="1:20" s="3" customFormat="1" x14ac:dyDescent="0.45">
       <c r="A281" s="7" t="s">
         <v>682</v>
       </c>
@@ -11062,7 +11133,7 @@
       <c r="S281"/>
       <c r="T281"/>
     </row>
-    <row r="282" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="282" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A282" s="7" t="s">
         <v>685</v>
       </c>
@@ -11085,7 +11156,7 @@
       <c r="I282" s="4"/>
       <c r="J282" s="4"/>
     </row>
-    <row r="283" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="283" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A283" s="7" t="s">
         <v>688</v>
       </c>
@@ -11108,7 +11179,7 @@
       <c r="I283" s="3"/>
       <c r="J283" s="3"/>
     </row>
-    <row r="284" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="284" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A284" s="7" t="s">
         <v>695</v>
       </c>
@@ -11131,7 +11202,7 @@
       <c r="I284" s="3"/>
       <c r="J284" s="3"/>
     </row>
-    <row r="285" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="285" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A285" s="7" t="s">
         <v>691</v>
       </c>
@@ -11151,7 +11222,7 @@
         <v>694</v>
       </c>
     </row>
-    <row r="286" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="286" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A286" s="7" t="s">
         <v>696</v>
       </c>
@@ -11174,7 +11245,7 @@
       <c r="I286" s="3"/>
       <c r="J286" s="3"/>
     </row>
-    <row r="287" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="287" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A287" s="7" t="s">
         <v>699</v>
       </c>
@@ -11194,7 +11265,7 @@
         <v>701</v>
       </c>
     </row>
-    <row r="288" spans="1:20" ht="30" x14ac:dyDescent="0.25">
+    <row r="288" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A288" s="7" t="s">
         <v>702</v>
       </c>
@@ -11214,7 +11285,7 @@
         <v>704</v>
       </c>
     </row>
-    <row r="289" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="289" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A289" s="7" t="s">
         <v>705</v>
       </c>
@@ -11234,7 +11305,7 @@
         <v>706</v>
       </c>
     </row>
-    <row r="290" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="290" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A290" s="7" t="s">
         <v>707</v>
       </c>
@@ -11254,7 +11325,7 @@
         <v>249</v>
       </c>
     </row>
-    <row r="291" spans="1:20" s="3" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="291" spans="1:20" s="3" customFormat="1" x14ac:dyDescent="0.45">
       <c r="A291" s="7" t="s">
         <v>709</v>
       </c>
@@ -11288,7 +11359,7 @@
       <c r="S291"/>
       <c r="T291"/>
     </row>
-    <row r="292" spans="1:20" s="3" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="292" spans="1:20" s="3" customFormat="1" x14ac:dyDescent="0.45">
       <c r="A292" s="7" t="s">
         <v>1037</v>
       </c>
@@ -11322,7 +11393,7 @@
       <c r="S292"/>
       <c r="T292"/>
     </row>
-    <row r="293" spans="1:20" ht="30" x14ac:dyDescent="0.25">
+    <row r="293" spans="1:20" ht="28.5" x14ac:dyDescent="0.45">
       <c r="A293" s="7" t="s">
         <v>1039</v>
       </c>
@@ -11342,7 +11413,7 @@
         <v>1121</v>
       </c>
     </row>
-    <row r="294" spans="1:20" s="3" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="294" spans="1:20" s="3" customFormat="1" x14ac:dyDescent="0.45">
       <c r="A294" s="7" t="s">
         <v>712</v>
       </c>
@@ -11376,7 +11447,7 @@
       <c r="S294"/>
       <c r="T294"/>
     </row>
-    <row r="295" spans="1:20" s="5" customFormat="1" ht="30" x14ac:dyDescent="0.25">
+    <row r="295" spans="1:20" s="5" customFormat="1" ht="28.5" x14ac:dyDescent="0.45">
       <c r="A295" s="7" t="s">
         <v>1041</v>
       </c>
@@ -11408,7 +11479,7 @@
       <c r="S295"/>
       <c r="T295"/>
     </row>
-    <row r="296" spans="1:20" s="3" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="296" spans="1:20" s="3" customFormat="1" x14ac:dyDescent="0.45">
       <c r="A296" s="7" t="s">
         <v>1042</v>
       </c>
@@ -11440,7 +11511,7 @@
       <c r="S296"/>
       <c r="T296"/>
     </row>
-    <row r="297" spans="1:20" s="5" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="297" spans="1:20" s="5" customFormat="1" x14ac:dyDescent="0.45">
       <c r="A297" s="7" t="s">
         <v>1044</v>
       </c>
@@ -11472,7 +11543,7 @@
       <c r="S297"/>
       <c r="T297"/>
     </row>
-    <row r="298" spans="1:20" s="5" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="298" spans="1:20" s="5" customFormat="1" x14ac:dyDescent="0.45">
       <c r="A298" s="7" t="s">
         <v>1046</v>
       </c>
@@ -11506,7 +11577,7 @@
       <c r="S298"/>
       <c r="T298"/>
     </row>
-    <row r="299" spans="1:20" s="3" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="299" spans="1:20" s="3" customFormat="1" x14ac:dyDescent="0.45">
       <c r="A299" s="7" t="s">
         <v>1048</v>
       </c>
@@ -11538,7 +11609,7 @@
       <c r="S299"/>
       <c r="T299"/>
     </row>
-    <row r="300" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="300" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A300" s="7" t="s">
         <v>1050</v>
       </c>
@@ -11568,7 +11639,7 @@
       <c r="S300" s="3"/>
       <c r="T300" s="3"/>
     </row>
-    <row r="301" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="301" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A301" s="7" t="s">
         <v>716</v>
       </c>
@@ -11588,7 +11659,7 @@
         <v>718</v>
       </c>
     </row>
-    <row r="302" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="302" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A302" s="7" t="s">
         <v>719</v>
       </c>
@@ -11608,7 +11679,7 @@
         <v>722</v>
       </c>
     </row>
-    <row r="303" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="303" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A303" s="7" t="s">
         <v>723</v>
       </c>
@@ -11634,7 +11705,7 @@
         <v>1132</v>
       </c>
     </row>
-    <row r="304" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="304" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A304" s="7" t="s">
         <v>727</v>
       </c>
@@ -11660,7 +11731,7 @@
         <v>1134</v>
       </c>
     </row>
-    <row r="305" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="305" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A305" s="7" t="s">
         <v>731</v>
       </c>
@@ -11685,7 +11756,7 @@
       </c>
       <c r="J305" s="5"/>
     </row>
-    <row r="306" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="306" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A306" s="7" t="s">
         <v>734</v>
       </c>
@@ -11708,7 +11779,7 @@
       <c r="I306" s="5"/>
       <c r="J306" s="5"/>
     </row>
-    <row r="307" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="307" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A307" s="7" t="s">
         <v>737</v>
       </c>
@@ -11728,7 +11799,7 @@
         <v>738</v>
       </c>
     </row>
-    <row r="308" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="308" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A308" s="7" t="s">
         <v>739</v>
       </c>
@@ -11751,7 +11822,7 @@
         <v>1139</v>
       </c>
     </row>
-    <row r="309" spans="1:20" s="3" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="309" spans="1:20" s="3" customFormat="1" x14ac:dyDescent="0.45">
       <c r="A309" s="7" t="s">
         <v>743</v>
       </c>
@@ -11785,7 +11856,7 @@
       <c r="S309"/>
       <c r="T309"/>
     </row>
-    <row r="310" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="310" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A310" s="7" t="s">
         <v>1055</v>
       </c>
@@ -11805,7 +11876,7 @@
         <v>747</v>
       </c>
     </row>
-    <row r="311" spans="1:20" s="3" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="311" spans="1:20" s="3" customFormat="1" x14ac:dyDescent="0.45">
       <c r="A311" s="7" t="s">
         <v>748</v>
       </c>
@@ -11839,7 +11910,7 @@
       <c r="S311" s="5"/>
       <c r="T311" s="5"/>
     </row>
-    <row r="312" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="312" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A312" s="7" t="s">
         <v>750</v>
       </c>
@@ -11866,7 +11937,7 @@
       <c r="S312" s="3"/>
       <c r="T312" s="3"/>
     </row>
-    <row r="313" spans="1:20" s="3" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="313" spans="1:20" s="3" customFormat="1" x14ac:dyDescent="0.45">
       <c r="A313" s="7" t="s">
         <v>753</v>
       </c>
@@ -11902,7 +11973,7 @@
       <c r="S313"/>
       <c r="T313"/>
     </row>
-    <row r="314" spans="1:20" ht="30" x14ac:dyDescent="0.25">
+    <row r="314" spans="1:20" ht="28.5" x14ac:dyDescent="0.45">
       <c r="A314" s="7" t="s">
         <v>757</v>
       </c>
@@ -11919,7 +11990,7 @@
         <v>89.13</v>
       </c>
     </row>
-    <row r="315" spans="1:20" s="3" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="315" spans="1:20" s="3" customFormat="1" x14ac:dyDescent="0.45">
       <c r="A315" s="7" t="s">
         <v>760</v>
       </c>
@@ -11947,7 +12018,7 @@
       <c r="I315" s="4"/>
       <c r="J315" s="4"/>
     </row>
-    <row r="316" spans="1:20" s="3" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="316" spans="1:20" s="3" customFormat="1" x14ac:dyDescent="0.45">
       <c r="A316" s="7" t="s">
         <v>1058</v>
       </c>
@@ -11979,7 +12050,7 @@
       <c r="S316" s="5"/>
       <c r="T316" s="5"/>
     </row>
-    <row r="317" spans="1:20" s="3" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="317" spans="1:20" s="3" customFormat="1" x14ac:dyDescent="0.45">
       <c r="A317" s="7" t="s">
         <v>1061</v>
       </c>
@@ -12011,7 +12082,7 @@
       <c r="S317" s="6"/>
       <c r="T317" s="6"/>
     </row>
-    <row r="318" spans="1:20" s="3" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="318" spans="1:20" s="3" customFormat="1" x14ac:dyDescent="0.45">
       <c r="A318" s="7" t="s">
         <v>1063</v>
       </c>
@@ -12043,7 +12114,7 @@
       <c r="S318" s="6"/>
       <c r="T318" s="6"/>
     </row>
-    <row r="319" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="319" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A319" s="7" t="s">
         <v>1066</v>
       </c>
@@ -12070,7 +12141,7 @@
       <c r="S319" s="6"/>
       <c r="T319" s="6"/>
     </row>
-    <row r="320" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="320" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A320" s="7" t="s">
         <v>763</v>
       </c>
@@ -12100,7 +12171,7 @@
       <c r="S320" s="6"/>
       <c r="T320" s="6"/>
     </row>
-    <row r="321" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="321" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A321" s="7" t="s">
         <v>767</v>
       </c>
@@ -12120,7 +12191,7 @@
         <v>770</v>
       </c>
     </row>
-    <row r="322" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="322" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A322" s="7" t="s">
         <v>771</v>
       </c>
@@ -12143,7 +12214,7 @@
         <v>1139</v>
       </c>
     </row>
-    <row r="323" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="323" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A323" s="7" t="s">
         <v>775</v>
       </c>
@@ -12163,7 +12234,7 @@
         <v>778</v>
       </c>
     </row>
-    <row r="324" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="324" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A324" s="7" t="s">
         <v>779</v>
       </c>
@@ -12186,7 +12257,7 @@
         <v>1139</v>
       </c>
     </row>
-    <row r="325" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="325" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A325" s="7" t="s">
         <v>782</v>
       </c>
@@ -12206,7 +12277,7 @@
         <v>783</v>
       </c>
     </row>
-    <row r="326" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="326" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A326" s="7" t="s">
         <v>784</v>
       </c>
@@ -12226,7 +12297,7 @@
         <v>785</v>
       </c>
     </row>
-    <row r="327" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="327" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A327" s="7" t="s">
         <v>786</v>
       </c>
@@ -12246,7 +12317,7 @@
         <v>787</v>
       </c>
     </row>
-    <row r="328" spans="1:20" s="3" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="328" spans="1:20" s="3" customFormat="1" x14ac:dyDescent="0.45">
       <c r="A328" s="7" t="s">
         <v>788</v>
       </c>
@@ -12280,7 +12351,7 @@
       <c r="S328"/>
       <c r="T328"/>
     </row>
-    <row r="329" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="329" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A329" s="7" t="s">
         <v>1073</v>
       </c>
@@ -12297,7 +12368,7 @@
         <v>203.15</v>
       </c>
     </row>
-    <row r="330" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="330" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A330" s="7" t="s">
         <v>790</v>
       </c>
@@ -12330,7 +12401,7 @@
       <c r="S330" s="3"/>
       <c r="T330" s="3"/>
     </row>
-    <row r="331" spans="1:20" s="3" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="331" spans="1:20" s="3" customFormat="1" x14ac:dyDescent="0.45">
       <c r="A331" s="7" t="s">
         <v>794</v>
       </c>
@@ -12360,7 +12431,7 @@
       <c r="S331"/>
       <c r="T331"/>
     </row>
-    <row r="332" spans="1:20" s="3" customFormat="1" ht="30" x14ac:dyDescent="0.25">
+    <row r="332" spans="1:20" s="3" customFormat="1" ht="28.5" x14ac:dyDescent="0.45">
       <c r="A332" s="7" t="s">
         <v>796</v>
       </c>
@@ -12394,7 +12465,7 @@
       <c r="S332"/>
       <c r="T332"/>
     </row>
-    <row r="333" spans="1:20" s="3" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="333" spans="1:20" s="3" customFormat="1" x14ac:dyDescent="0.45">
       <c r="A333" s="7" t="s">
         <v>798</v>
       </c>
@@ -12424,7 +12495,7 @@
       <c r="S333"/>
       <c r="T333"/>
     </row>
-    <row r="334" spans="1:20" s="3" customFormat="1" ht="30" x14ac:dyDescent="0.25">
+    <row r="334" spans="1:20" s="3" customFormat="1" x14ac:dyDescent="0.45">
       <c r="A334" s="7" t="s">
         <v>800</v>
       </c>
@@ -12456,7 +12527,7 @@
       <c r="S334"/>
       <c r="T334"/>
     </row>
-    <row r="335" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="335" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A335" s="7" t="s">
         <v>802</v>
       </c>
@@ -12486,7 +12557,7 @@
       <c r="S335" s="3"/>
       <c r="T335" s="3"/>
     </row>
-    <row r="336" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="336" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A336" s="7" t="s">
         <v>805</v>
       </c>
@@ -12516,7 +12587,7 @@
       <c r="S336" s="3"/>
       <c r="T336" s="3"/>
     </row>
-    <row r="337" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="337" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A337" s="7" t="s">
         <v>807</v>
       </c>
@@ -12549,7 +12620,7 @@
       <c r="S337" s="3"/>
       <c r="T337" s="3"/>
     </row>
-    <row r="338" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="338" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A338" s="7" t="s">
         <v>809</v>
       </c>
@@ -12579,7 +12650,7 @@
       <c r="S338" s="3"/>
       <c r="T338" s="3"/>
     </row>
-    <row r="339" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="339" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A339" s="7" t="s">
         <v>812</v>
       </c>
@@ -12599,7 +12670,7 @@
         <v>814</v>
       </c>
     </row>
-    <row r="340" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="340" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A340" s="7" t="s">
         <v>1076</v>
       </c>
@@ -12619,7 +12690,7 @@
         <v>1103</v>
       </c>
     </row>
-    <row r="341" spans="1:20" s="3" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="341" spans="1:20" s="3" customFormat="1" x14ac:dyDescent="0.45">
       <c r="A341" s="7" t="s">
         <v>1079</v>
       </c>
@@ -12647,7 +12718,7 @@
       <c r="S341"/>
       <c r="T341"/>
     </row>
-    <row r="342" spans="1:20" s="3" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="342" spans="1:20" s="3" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A342" s="7" t="s">
         <v>1080</v>
       </c>
@@ -12671,7 +12742,7 @@
       </c>
       <c r="J342"/>
     </row>
-    <row r="343" spans="1:20" s="3" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="343" spans="1:20" s="3" customFormat="1" x14ac:dyDescent="0.45">
       <c r="A343" s="7" t="s">
         <v>1082</v>
       </c>
@@ -12695,7 +12766,7 @@
       </c>
       <c r="J343"/>
     </row>
-    <row r="344" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="344" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A344" s="7" t="s">
         <v>815</v>
       </c>
@@ -12715,7 +12786,7 @@
         <v>818</v>
       </c>
     </row>
-    <row r="345" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="345" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A345" s="7" t="s">
         <v>819</v>
       </c>
@@ -12735,7 +12806,7 @@
         <v>822</v>
       </c>
     </row>
-    <row r="346" spans="1:20" s="3" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="346" spans="1:20" s="3" customFormat="1" x14ac:dyDescent="0.45">
       <c r="A346" s="7" t="s">
         <v>823</v>
       </c>
@@ -12757,7 +12828,7 @@
       <c r="I346"/>
       <c r="J346"/>
     </row>
-    <row r="347" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="347" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A347" s="7" t="s">
         <v>825</v>
       </c>
@@ -12777,7 +12848,7 @@
         <v>828</v>
       </c>
     </row>
-    <row r="348" spans="1:20" s="3" customFormat="1" ht="30" x14ac:dyDescent="0.25">
+    <row r="348" spans="1:20" s="3" customFormat="1" x14ac:dyDescent="0.45">
       <c r="A348" s="7" t="s">
         <v>1084</v>
       </c>
@@ -12803,36 +12874,66 @@
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:J348">
     <sortCondition ref="A2:A348"/>
   </sortState>
-  <conditionalFormatting sqref="A2:Y500">
-    <cfRule type="expression" dxfId="8" priority="10">
+  <conditionalFormatting sqref="A184:Y500 A2:Y181 A182:C183 E182:Y183 D182">
+    <cfRule type="expression" dxfId="17" priority="28">
       <formula>AND(MOD(ROW(),2)=0,$I2&lt;&gt;"")</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="7" priority="11">
+    <cfRule type="expression" dxfId="16" priority="29">
       <formula>AND(MOD(ROW(),1)=0,$I2&lt;&gt;"")</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="6" priority="12">
+    <cfRule type="expression" dxfId="15" priority="30">
       <formula>AND(MOD(ROW(),2)=0,LOWER($B2)="false")</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="5" priority="13">
+    <cfRule type="expression" dxfId="14" priority="31">
       <formula>AND(MOD(ROW(),2)=1,LOWER($B2)="false")</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="4" priority="14">
+    <cfRule type="expression" dxfId="13" priority="32">
       <formula>AND(MOD(ROW(),2)=0,LOWER($B2)="idk")</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="3" priority="15">
+    <cfRule type="expression" dxfId="12" priority="33">
       <formula>AND(MOD(ROW(),2)=1,LOWER($B2)="idk")</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="2" priority="16">
+    <cfRule type="expression" dxfId="11" priority="34">
       <formula>AND(MOD(ROW(),2)=0,LOWER($B2)="true")</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="1" priority="17">
+    <cfRule type="expression" dxfId="10" priority="35">
       <formula>AND(MOD(ROW(),2)=1,LOWER($B2)="true")</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="0" priority="18">
+    <cfRule type="expression" dxfId="9" priority="36">
+      <formula>MOD(ROW(),2)=0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="D183">
+    <cfRule type="expression" dxfId="8" priority="1">
+      <formula>AND(MOD(ROW(),2)=0,$I183&lt;&gt;"")</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="7" priority="2">
+      <formula>AND(MOD(ROW(),1)=0,$I183&lt;&gt;"")</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="6" priority="3">
+      <formula>AND(MOD(ROW(),2)=0,LOWER($B183)="false")</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="5" priority="4">
+      <formula>AND(MOD(ROW(),2)=1,LOWER($B183)="false")</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="4" priority="5">
+      <formula>AND(MOD(ROW(),2)=0,LOWER($B183)="idk")</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="3" priority="6">
+      <formula>AND(MOD(ROW(),2)=1,LOWER($B183)="idk")</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="2" priority="7">
+      <formula>AND(MOD(ROW(),2)=0,LOWER($B183)="true")</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="1" priority="8">
+      <formula>AND(MOD(ROW(),2)=1,LOWER($B183)="true")</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="0" priority="9">
       <formula>MOD(ROW(),2)=0</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" verticalDpi="0" r:id="rId1"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
       <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="2">
@@ -12857,32 +12958,32 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BE476A99-88D9-4674-8BF6-BFC09110212C}">
   <dimension ref="A1:A6"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="1" max="1" width="9.140625" style="10"/>
+    <col min="1" max="1" width="9.1328125" style="10"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A1" s="10" t="s">
         <v>1108</v>
       </c>
     </row>
-    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A3" s="10" t="s">
         <v>1110</v>
       </c>
     </row>
-    <row r="4" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A4" s="10" t="s">
         <v>1106</v>
       </c>
     </row>
-    <row r="5" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A5" s="10" t="s">
         <v>1109</v>
       </c>
     </row>
-    <row r="6" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A6" s="10" t="s">
         <v>1111</v>
       </c>

</xml_diff>